<commit_message>
refactor: remove Selected scenario callout from Scenarios sheet
Drops the CHOOSE()-based summary block below the three-scenario table.
scenario_switch on the Assumptions sheet was its only consumer and is
now an orphaned input with no formula referencing it.
</commit_message>
<xml_diff>
--- a/workbook/tutoring-financial-model.xlsx
+++ b/workbook/tutoring-financial-model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\tutoring-financial-model\workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F98863-97A7-4BFD-A9BA-251961465D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E2C88F-12A6-49E3-B033-305BA3677B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="250">
   <si>
     <t>Tutoring Business Financial Model</t>
   </si>
@@ -773,12 +773,6 @@
   </si>
   <si>
     <t>Net income (annualised, $)</t>
-  </si>
-  <si>
-    <t>Selected scenario (Assumptions!scenario_switch)</t>
-  </si>
-  <si>
-    <t>Selected scenario net income ($)</t>
   </si>
   <si>
     <t>Sensitivity: net income by rate × utilisation</t>
@@ -10262,7 +10256,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -10448,24 +10442,6 @@
       <c r="D13" s="24">
         <f>D9-D10-D12</f>
         <v>32754.399999999994</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="25" t="s">
-        <v>244</v>
-      </c>
-      <c r="B15" s="20" t="str">
-        <f>CHOOSE(Assumptions!$B$35,B4,C4,D4)</f>
-        <v>1. Base (actual)</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
-        <v>245</v>
-      </c>
-      <c r="B16" s="24">
-        <f>CHOOSE(Assumptions!$B$35,B13,C13,D13)</f>
-        <v>30682.400000000001</v>
       </c>
     </row>
   </sheetData>
@@ -10489,7 +10465,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="34" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B1" s="31"/>
       <c r="C1" s="31"/>
@@ -10500,7 +10476,7 @@
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B2" s="31"/>
       <c r="C2" s="31"/>
@@ -10511,7 +10487,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="27" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B4" s="19">
         <f>'P&amp;L and provisioning'!$B$15</f>
@@ -10520,7 +10496,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="27" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B5" s="19">
         <f>ABS('P&amp;L and provisioning'!$B$16)</f>
@@ -10529,7 +10505,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="28">
@@ -10550,7 +10526,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B8" s="29">
         <v>0.8</v>

</xml_diff>

<commit_message>
fix: align Annualisation factor row with rest of P&L table
Shortened the wrapped label (which forced a taller row than its
neighbours) and moved the working-weeks/weeks-per-term derivation into
the notes column, matching how the Tax provision row already uses it.
</commit_message>
<xml_diff>
--- a/workbook/tutoring-financial-model.xlsx
+++ b/workbook/tutoring-financial-model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\tutoring-financial-model\workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E2C88F-12A6-49E3-B033-305BA3677B33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F36971A-E7E4-4E37-A7D4-B09677DDA6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1227" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="251">
   <si>
     <t>Tutoring Business Financial Model</t>
   </si>
@@ -727,7 +727,10 @@
     <t>Annualised run-rate (extrapolated, NOT an actual full-year figure; the business wound up ~18 Sept 2026)</t>
   </si>
   <si>
-    <t>Annualisation factor (working weeks/yr ÷ weeks/term)</t>
+    <t>Annualisation factor</t>
+  </si>
+  <si>
+    <t>Working weeks/yr ÷ weeks/term.</t>
   </si>
   <si>
     <t>Net income (annualised)</t>
@@ -913,7 +916,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -950,9 +953,6 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1321,10 +1321,10 @@
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="31"/>
+      <c r="B8" s="30"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -1377,10 +1377,10 @@
       </c>
     </row>
     <row r="21" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="31"/>
+      <c r="B21" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1427,12 +1427,12 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
     </row>
     <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -1478,12 +1478,12 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
@@ -1514,12 +1514,12 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="32" t="s">
+      <c r="A15" s="31" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="31"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
@@ -1608,12 +1608,12 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
     </row>
     <row r="24" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
@@ -1746,12 +1746,12 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="32" t="s">
+      <c r="A34" s="31" t="s">
         <v>80</v>
       </c>
-      <c r="B34" s="31"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="31"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
     </row>
     <row r="35" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
@@ -1833,22 +1833,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -7547,14 +7547,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>182</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -8546,28 +8546,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>190</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="4" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
@@ -9920,18 +9920,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
         <v>199</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -10079,18 +10079,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="33" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="34" t="s">
         <v>218</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="37"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="36"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -10165,21 +10165,23 @@
       <c r="C10" s="9"/>
     </row>
     <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="35" t="s">
+      <c r="A13" s="34" t="s">
         <v>227</v>
       </c>
-      <c r="B13" s="36"/>
-      <c r="C13" s="37"/>
-    </row>
-    <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="26" t="s">
+      <c r="B13" s="35"/>
+      <c r="C13" s="36"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>228</v>
       </c>
       <c r="B14" s="14">
         <f>Assumptions!$B$18/Assumptions!$B$17</f>
         <v>4</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="9" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
@@ -10237,7 +10239,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B21" s="24">
         <f t="shared" si="0"/>
@@ -10264,36 +10266,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
-        <v>230</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="A1" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="2" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
-        <v>231</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
+      <c r="A2" s="32" t="s">
+        <v>232</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
     </row>
     <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B5" s="14">
         <f>Capacity!$B$10</f>
@@ -10310,7 +10312,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B6" s="7">
         <f>Assumptions!$B$7</f>
@@ -10327,7 +10329,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B7" s="24">
         <f>B5*Assumptions!$B$18*B6</f>
@@ -10344,7 +10346,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B8" s="7">
         <f>Assumptions!$B$32*Assumptions!$B$18</f>
@@ -10361,7 +10363,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B9" s="24">
         <f>B7-B8</f>
@@ -10378,7 +10380,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B10" s="7">
         <f>B9*Assumptions!$B$12</f>
@@ -10395,7 +10397,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B11" s="7">
         <f>B9-B10</f>
@@ -10412,7 +10414,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B12" s="7">
         <f>B11*Assumptions!$B$13</f>
@@ -10429,7 +10431,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B13" s="24">
         <f>B9-B10-B12</f>
@@ -10464,30 +10466,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
+      <c r="A1" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
-        <v>245</v>
-      </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
+      <c r="A2" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="27" t="s">
-        <v>246</v>
+      <c r="A4" s="26" t="s">
+        <v>247</v>
       </c>
       <c r="B4" s="19">
         <f>'P&amp;L and provisioning'!$B$15</f>
@@ -10495,8 +10497,8 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
-        <v>247</v>
+      <c r="A5" s="26" t="s">
+        <v>248</v>
       </c>
       <c r="B5" s="19">
         <f>ABS('P&amp;L and provisioning'!$B$16)</f>
@@ -10505,30 +10507,30 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="C7" s="28">
+      <c r="C7" s="27">
         <v>0.9</v>
       </c>
-      <c r="D7" s="28">
+      <c r="D7" s="27">
         <v>0.95</v>
       </c>
-      <c r="E7" s="28">
+      <c r="E7" s="27">
         <v>1</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="27">
         <v>1.05</v>
       </c>
-      <c r="G7" s="28">
+      <c r="G7" s="27">
         <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="38" t="s">
-        <v>249</v>
-      </c>
-      <c r="B8" s="29">
+      <c r="A8" s="37" t="s">
+        <v>250</v>
+      </c>
+      <c r="B8" s="28">
         <v>0.8</v>
       </c>
       <c r="C8" s="7">
@@ -10553,8 +10555,8 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="31"/>
-      <c r="B9" s="29">
+      <c r="A9" s="30"/>
+      <c r="B9" s="28">
         <v>0.9</v>
       </c>
       <c r="C9" s="7">
@@ -10579,8 +10581,8 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="31"/>
-      <c r="B10" s="29">
+      <c r="A10" s="30"/>
+      <c r="B10" s="28">
         <v>1</v>
       </c>
       <c r="C10" s="7">
@@ -10605,8 +10607,8 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="31"/>
-      <c r="B11" s="29">
+      <c r="A11" s="30"/>
+      <c r="B11" s="28">
         <v>1.1000000000000001</v>
       </c>
       <c r="C11" s="7">
@@ -10631,8 +10633,8 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="31"/>
-      <c r="B12" s="29">
+      <c r="A12" s="30"/>
+      <c r="B12" s="28">
         <v>1.2</v>
       </c>
       <c r="C12" s="7">

</xml_diff>

<commit_message>
refactor: simplify P&L annualised run-rate table
Shorten the banner to "Annualised run-rate" and move the extrapolation/
wind-up caveat to a visible note under the table instead. Drop the
now near-empty notes column from this table, moving the annualisation
factor's derivation to a cell comment on its value cell.
</commit_message>
<xml_diff>
--- a/workbook/tutoring-financial-model.xlsx
+++ b/workbook/tutoring-financial-model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\tutoring-financial-model\workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F36971A-E7E4-4E37-A7D4-B09677DDA6D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{426B7F9A-F5FC-43CD-95FD-456ED8511B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,8 +40,32 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Model</author>
+  </authors>
+  <commentList>
+    <comment ref="B14" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0600-000001000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Working weeks/yr ÷ weeks/term.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="250">
   <si>
     <t>Tutoring Business Financial Model</t>
   </si>
@@ -724,13 +748,10 @@
     <t>Net income (period)</t>
   </si>
   <si>
-    <t>Annualised run-rate (extrapolated, NOT an actual full-year figure; the business wound up ~18 Sept 2026)</t>
+    <t>Annualised run-rate</t>
   </si>
   <si>
     <t>Annualisation factor</t>
-  </si>
-  <si>
-    <t>Working weeks/yr ÷ weeks/term.</t>
   </si>
   <si>
     <t>Net income (annualised)</t>
@@ -972,8 +993,8 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -10069,8 +10090,8 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:C21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -10089,8 +10110,8 @@
       <c r="A3" s="34" t="s">
         <v>218</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="36"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="35"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
@@ -10164,12 +10185,11 @@
       </c>
       <c r="C10" s="9"/>
     </row>
-    <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="34" t="s">
         <v>227</v>
       </c>
       <c r="B13" s="35"/>
-      <c r="C13" s="36"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
@@ -10179,9 +10199,6 @@
         <f>Assumptions!$B$18/Assumptions!$B$17</f>
         <v>4</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>229</v>
-      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
@@ -10239,20 +10256,28 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B21" s="24">
         <f t="shared" si="0"/>
         <v>30682.400000000001</v>
       </c>
     </row>
+    <row r="23" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="B23" s="30"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A23:B23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10267,7 +10292,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -10275,7 +10300,7 @@
     </row>
     <row r="2" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
@@ -10284,18 +10309,18 @@
     <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B5" s="14">
         <f>Capacity!$B$10</f>
@@ -10312,7 +10337,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B6" s="7">
         <f>Assumptions!$B$7</f>
@@ -10329,7 +10354,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B7" s="24">
         <f>B5*Assumptions!$B$18*B6</f>
@@ -10346,7 +10371,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B8" s="7">
         <f>Assumptions!$B$32*Assumptions!$B$18</f>
@@ -10363,7 +10388,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B9" s="24">
         <f>B7-B8</f>
@@ -10380,7 +10405,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B10" s="7">
         <f>B9*Assumptions!$B$12</f>
@@ -10397,7 +10422,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B11" s="7">
         <f>B9-B10</f>
@@ -10414,7 +10439,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B12" s="7">
         <f>B11*Assumptions!$B$13</f>
@@ -10431,7 +10456,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="21" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B13" s="24">
         <f>B9-B10-B12</f>
@@ -10467,7 +10492,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
@@ -10478,7 +10503,7 @@
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
@@ -10489,7 +10514,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B4" s="19">
         <f>'P&amp;L and provisioning'!$B$15</f>
@@ -10498,7 +10523,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B5" s="19">
         <f>ABS('P&amp;L and provisioning'!$B$16)</f>
@@ -10507,7 +10532,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="27">
@@ -10528,7 +10553,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="37" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B8" s="28">
         <v>0.8</v>

</xml_diff>